<commit_message>
Filter and XLookup Data
</commit_message>
<xml_diff>
--- a/Excel/ConditionalFormat.xlsx
+++ b/Excel/ConditionalFormat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_AF\DPBA_D2957\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27DABF5-2A4F-482A-A13B-F523EBB8354F}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A48A35-5FC2-4BAF-80C1-FB633909CBC9}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7240" firstSheet="4" activeTab="11" xr2:uid="{0C51D57F-E629-49C9-8C56-ABCE15FC41BE}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7240" firstSheet="1" activeTab="10" xr2:uid="{0C51D57F-E629-49C9-8C56-ABCE15FC41BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Intro" sheetId="1" r:id="rId1"/>
@@ -579,7 +579,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$-14009]dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-14009]dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -753,26 +753,14 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="21">
     <dxf>
       <font>
         <b/>
@@ -1002,102 +990,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2873,12 +2765,12 @@
   </sheetData>
   <dataConsolidate/>
   <conditionalFormatting sqref="J2 A4:C99">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$A2=$G$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D4:D99">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$A4=$G$2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4310,7 +4202,7 @@
   </sortState>
   <dataConsolidate/>
   <conditionalFormatting sqref="A4:D99">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND($A4=$G$2,$D4&gt;=$H$2)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5745,7 +5637,7 @@
   </sheetData>
   <dataConsolidate/>
   <conditionalFormatting sqref="A4:D99">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND($A4=$G$2,AND($D4&gt;=$H$2,$D4&lt;=$I$2))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5999,26 +5891,26 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H7:H16">
-    <cfRule type="cellIs" dxfId="21" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="4" operator="equal">
       <formula>"cHENNAI"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="5" operator="equal">
       <formula>"KolKATA"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J7:J16">
-    <cfRule type="cellIs" dxfId="19" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7:K16">
-    <cfRule type="cellIs" dxfId="18" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="17" priority="2" operator="between">
       <formula>4</formula>
       <formula>9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L7:L16">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6187,23 +6079,23 @@
     <sortCondition ref="H7"/>
   </sortState>
   <conditionalFormatting sqref="J7:J16">
-    <cfRule type="cellIs" dxfId="16" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="4" operator="greaterThan">
       <formula>500</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7:K16">
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="14" priority="3" operator="between">
       <formula>4</formula>
       <formula>9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L7:L16">
-    <cfRule type="cellIs" dxfId="14" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:H16">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="12" priority="1">
       <formula>EXACT($H7,$I$5)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7143,22 +7035,22 @@
     <sortCondition ref="F6"/>
   </sortState>
   <conditionalFormatting sqref="G6:G17">
-    <cfRule type="top10" dxfId="12" priority="6" rank="5"/>
+    <cfRule type="top10" dxfId="11" priority="6" rank="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H17">
-    <cfRule type="top10" dxfId="11" priority="5" bottom="1" rank="6"/>
+    <cfRule type="top10" dxfId="10" priority="5" bottom="1" rank="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:I17">
-    <cfRule type="aboveAverage" dxfId="10" priority="4"/>
+    <cfRule type="aboveAverage" dxfId="9" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J6:J17">
-    <cfRule type="aboveAverage" dxfId="9" priority="3" aboveAverage="0"/>
+    <cfRule type="aboveAverage" dxfId="8" priority="3" aboveAverage="0"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K17">
-    <cfRule type="top10" dxfId="8" priority="2" percent="1" rank="30"/>
+    <cfRule type="top10" dxfId="7" priority="2" percent="1" rank="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L6:L17">
-    <cfRule type="top10" dxfId="7" priority="1" percent="1" bottom="1" rank="50"/>
+    <cfRule type="top10" dxfId="6" priority="1" percent="1" bottom="1" rank="50"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8548,7 +8440,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A4:D99">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$A4=$G$2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9941,7 +9833,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A4:C99">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$A4=$G$2</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>